<commit_message>
Task 3: Frontend Testing - finished
</commit_message>
<xml_diff>
--- a/Exam/gymtrackerpro/app/(auth)/login/_components/__tests__/ft/login-form/login-form-ft-form.xlsx
+++ b/Exam/gymtrackerpro/app/(auth)/login/_components/__tests__/ft/login-form/login-form-ft-form.xlsx
@@ -13,9 +13,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="90">
-  <si>
-    <t>Component: LoginForm — LoginForm - renders a login form with email and password fields, runs client-side zod validation before calling the login server action, and redirects the user to their role-specific dashboard on success.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="127">
+  <si>
+    <t>Component: LoginForm — LoginForm - renders a login form, checks loginUserSchema client-side, calls the login server action only for valid inputs, and redirects by returned role.</t>
   </si>
   <si>
     <t/>
@@ -47,6 +47,7 @@
   <si>
     <t xml:space="preserve">Mock next/navigation: useRouter returns { push: jest.fn() }.
 Mock @/lib/controller/auth-controller: login is a jest.fn().
+Mock generated Prisma Role enum for jsdom compatibility.
 No providers required - the component uses no React context.</t>
   </si>
   <si>
@@ -56,40 +57,43 @@
     <t>Render Output</t>
   </si>
   <si>
-    <t xml:space="preserve">A &lt;form&gt; element.
-A &lt;label&gt; "Email" associated with an &lt;input id="email"&gt; of type email.
-A &lt;label&gt; "Password" associated with an &lt;input id="password"&gt; of type password.
-A &lt;button&gt; with accessible name "Sign in", enabled.
-No &lt;Alert&gt; visible (result is null on initial render).</t>
+    <t xml:space="preserve">A &lt;form noValidate&gt; element.
+A label "Email" associated with an email input.
+A label "Password" associated with a password input.
+An enabled submit button with accessible name "Sign in".
+No alert visible in the initial result=null state.</t>
   </si>
   <si>
     <t>Postcondition</t>
   </si>
   <si>
-    <t xml:space="preserve">login() called once with a valid LoginUserInput when zod validation passes.
-router.push("/admin/dashboard") called when login resolves with role ADMIN.
-router.push("/member/dashboard") called when login resolves with role MEMBER.
-router.push("/login") called when login resolves with an unrecognised role (switch default).
-login() NOT called when zod validation fails - early return fires before startTransition.
-Destructive Alert visible with server error message and button re-enabled when login returns success: false.</t>
+    <t xml:space="preserve">login() is not called when loginUserSchema.safeParse(inputs) fails.
+login() is called once with trimmed email and password when both schema predicates pass.
+router.push("/admin/dashboard") is called for role ADMIN.
+router.push("/member/dashboard") is called for role MEMBER.
+router.push("/login") is called for an unrecognised role.
+A failed server result renders its message and any returned field errors.</t>
   </si>
   <si>
     <t>Remarks</t>
   </si>
   <si>
-    <t>Run: npx jest login-form.test.tsx</t>
-  </si>
-  <si>
-    <t>isPending relies on React 19 async-transition support - startTransition(async fn) keeps isPending=true until the promise resolves.</t>
-  </si>
-  <si>
-    <t>jsdom does not enforce HTML5 browser validation (type="email", required); the zod safeParse in handleSubmit is the only validation gate tested here.</t>
-  </si>
-  <si>
-    <t>The switch statement has three branches (ADMIN, MEMBER, default) - each needs its own test case.</t>
-  </si>
-  <si>
-    <t>Field-level error text is generated by zod and depends on loginUserSchema - tests assert structural presence of error paragraphs, not exact messages.</t>
+    <t>Run: npx jest app/\(auth\)/login/_components/__tests__/ft/login-form/login-form.test.tsx --selectProjects jsdom</t>
+  </si>
+  <si>
+    <t>The test file intentionally has only the main describe("LoginForm") block.</t>
+  </si>
+  <si>
+    <t>Predicate coverage: email valid/invalid and password valid/invalid are covered as a four-combination truth table.</t>
+  </si>
+  <si>
+    <t>Password decision coverage includes min length, max length, uppercase, number, and special-character constraints.</t>
+  </si>
+  <si>
+    <t>jsdom does not enforce browser validation because the form has noValidate; the zod safeParse branch is the validation gate.</t>
+  </si>
+  <si>
+    <t>React 19 async-transition support keeps isPending=true while the mocked login promise is unresolved.</t>
   </si>
   <si>
     <t>No TC</t>
@@ -113,20 +117,16 @@
     <t>TC-01</t>
   </si>
   <si>
-    <t>Renders email input, password input, and an enabled "Sign in" button with no alert visible in the default idle state.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mockLogin not configured (not called).
-render(&lt;LoginForm /&gt;)</t>
+    <t>Renders email input, password input, and enabled Sign in button with no alert in the default state.</t>
+  </si>
+  <si>
+    <t>render(&lt;LoginForm /&gt;); login mock not configured.</t>
   </si>
   <si>
     <t>No interaction - render only.</t>
   </si>
   <si>
-    <t xml:space="preserve">getByLabelText("Email") is in the document.
-getByLabelText("Password") is in the document.
-getByRole("button", {name: "Sign in"}) is in the document and is enabled.
-queryByRole("alert") returns null.</t>
+    <t>Email and Password inputs are visible; Sign in button is enabled; no alert is present.</t>
   </si>
   <si>
     <t>Passed</t>
@@ -135,156 +135,226 @@
     <t>TC-02</t>
   </si>
   <si>
-    <t>Submitting with both fields empty shows the destructive alert with "Validation failed" and does not call the login server action.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mockLogin not configured.
-render(&lt;LoginForm /&gt;)
-No input typed - both fields remain empty.</t>
-  </si>
-  <si>
-    <t>userEvent.click(getByRole("button", {name: "Sign in"}))</t>
-  </si>
-  <si>
-    <t xml:space="preserve">getByRole("alert") is in the document and contains text "Validation failed".
-mockLogin has not been called.</t>
+    <t>Email invalid and password invalid: empty fields show both field errors and skip login.</t>
+  </si>
+  <si>
+    <t>render(&lt;LoginForm /&gt;); leave Email and Password empty.</t>
+  </si>
+  <si>
+    <t>userEvent.click(Sign in)</t>
+  </si>
+  <si>
+    <t>Validation failed alert visible; Email and Password field errors visible; login not called.</t>
   </si>
   <si>
     <t>TC-03</t>
   </si>
   <si>
-    <t>Submitting with a valid email but an empty password triggers validation failure and does not call the login server action.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mockLogin not configured.
-render(&lt;LoginForm /&gt;)
-Type "test@example.com" into the Email input; leave Password empty.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">getByRole("alert") is in the document (validation failed).
-A &lt;p&gt; error element is visible adjacent to the Password input.
-No &lt;p&gt; error element is visible adjacent to the Email input.
-mockLogin has not been called.</t>
+    <t>Email valid and password invalid: shows only password error and skips login.</t>
+  </si>
+  <si>
+    <t>Type Email test@example.com and Password weakpass.</t>
+  </si>
+  <si>
+    <t>Validation failed alert visible; Password field error visible; Email field has no error; login not called.</t>
   </si>
   <si>
     <t>TC-04</t>
   </si>
   <si>
-    <t>Submitting with an invalid email format and a valid password triggers validation failure and does not call the login server action.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mockLogin not configured.
-render(&lt;LoginForm /&gt;)
-Type "not-an-email" into the Email input.
-Type "Password123!" into the Password input.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">getByRole("alert") is in the document (validation failed).
-A &lt;p&gt; error element is visible adjacent to the Email input.
-No &lt;p&gt; error element is visible adjacent to the Password input.
-mockLogin has not been called.</t>
+    <t>Email invalid and password valid: shows only email error and skips login.</t>
+  </si>
+  <si>
+    <t>Type Email not-an-email and Password Password123!.</t>
+  </si>
+  <si>
+    <t>Validation failed alert visible; Email field error visible; Password field has no error; login not called.</t>
   </si>
   <si>
     <t>TC-05</t>
   </si>
   <si>
-    <t>A successful login response with role ADMIN navigates to /admin/dashboard.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mockLogin.mockResolvedValueOnce({ success: true, data: { role: Role.ADMIN } }).
-render(&lt;LoginForm /&gt;)
-Type valid credentials into both fields.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mockLogin called once with { email: "test@example.com", password: "Password123!" }.
-mockPush called once with "/admin/dashboard".</t>
+    <t>Email invalid and password invalid: shows both field errors and skips login.</t>
+  </si>
+  <si>
+    <t>Type Email not-an-email and Password weakpass.</t>
+  </si>
+  <si>
+    <t>Validation failed alert visible; both field errors visible; login not called.</t>
   </si>
   <si>
     <t>TC-06</t>
   </si>
   <si>
-    <t>A successful login response with role MEMBER navigates to /member/dashboard.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mockLogin.mockResolvedValueOnce({ success: true, data: { role: Role.MEMBER } }).
-render(&lt;LoginForm /&gt;)
-Type valid credentials into both fields.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mockLogin called once.
-mockPush called once with "/member/dashboard".</t>
+    <t>Email valid and password valid: calls login once with trimmed email and valid password.</t>
+  </si>
+  <si>
+    <t>login resolves failed server result; type Email "  test@example.com  " and Password Password123!.</t>
+  </si>
+  <si>
+    <t>login called once with {email:"test@example.com", password:"Password123!"}.</t>
   </si>
   <si>
     <t>TC-07</t>
   </si>
   <si>
-    <t>A successful login response with an unrecognised role falls through the switch default and navigates to /login.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mockLogin.mockResolvedValueOnce({ success: true, data: { role: "UNKNOWN" as Role } }).
-render(&lt;LoginForm /&gt;)
-Type valid credentials into both fields.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mockLogin called once.
-mockPush called once with "/login".</t>
+    <t>Password length below minimum fails password predicate and skips login.</t>
+  </si>
+  <si>
+    <t>Type valid email and password P1@aaaa (7 characters).</t>
+  </si>
+  <si>
+    <t>Password min-length message visible; login not called.</t>
   </si>
   <si>
     <t>TC-08</t>
   </si>
   <si>
-    <t>When the login server action returns success: false the alert shows the server error message and the submit button is re-enabled.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mockLogin.mockResolvedValueOnce({ success: false, message: "Invalid credentials" }).
-render(&lt;LoginForm /&gt;)
-Type valid credentials into both fields.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">getByRole("alert") contains text "Invalid credentials".
-getByRole("button", {name: "Sign in"}) is enabled.
-mockPush has not been called.</t>
+    <t>Password length above maximum fails password predicate and skips login.</t>
+  </si>
+  <si>
+    <t>Type valid email and a 65-character password beginning with P1@.</t>
+  </si>
+  <si>
+    <t>Password max-length message visible; login not called.</t>
   </si>
   <si>
     <t>TC-09</t>
   </si>
   <si>
-    <t>While the login action is in flight the submit button is disabled and its label changes to "Signing in…".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mockLogin set to a manually-controlled promise that does not resolve during the assertion.
-render(&lt;LoginForm /&gt;)
-Type valid credentials into both fields.</t>
-  </si>
-  <si>
-    <t>userEvent.click(button) - do not resolve the login promise before asserting.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">getByRole("button") is disabled.
-getByText("Signing in…") is in the document.
-queryByText("Sign in") is not in the document.</t>
+    <t>Password missing uppercase fails password predicate and skips login.</t>
+  </si>
+  <si>
+    <t>Type valid email and password password123!.</t>
+  </si>
+  <si>
+    <t>Uppercase-character password message visible; login not called.</t>
   </si>
   <si>
     <t>TC-10</t>
   </si>
   <si>
-    <t>After a server-side failure the user can resubmit and a subsequent valid submission succeeds.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mockLogin configured with two sequential return values:
-  1. { success: false, message: "Invalid credentials" }
-  2. { success: true, data: { role: Role.MEMBER } }
-render(&lt;LoginForm /&gt;)
-Type valid credentials into both fields.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">First click - awaited, produces failure.
-Second click - awaited, produces success.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">After first click: alert with "Invalid credentials" is visible.
-After second click: mockPush called with "/member/dashboard".
-mockLogin called exactly twice in total.</t>
+    <t>Password missing number fails password predicate and skips login.</t>
+  </si>
+  <si>
+    <t>Type valid email and password Password!.</t>
+  </si>
+  <si>
+    <t>Number password message visible; login not called.</t>
+  </si>
+  <si>
+    <t>TC-11</t>
+  </si>
+  <si>
+    <t>Password missing special character fails password predicate and skips login.</t>
+  </si>
+  <si>
+    <t>Type valid email and password Password123.</t>
+  </si>
+  <si>
+    <t>Special-character password message visible; login not called.</t>
+  </si>
+  <si>
+    <t>TC-12</t>
+  </si>
+  <si>
+    <t>Successful login with ADMIN role navigates to admin dashboard.</t>
+  </si>
+  <si>
+    <t>login resolves {success:true,data:{role:Role.ADMIN}}; type valid credentials.</t>
+  </si>
+  <si>
+    <t>login called once with valid credentials; router.push called with /admin/dashboard.</t>
+  </si>
+  <si>
+    <t>TC-13</t>
+  </si>
+  <si>
+    <t>Successful login with MEMBER role navigates to member dashboard.</t>
+  </si>
+  <si>
+    <t>login resolves {success:true,data:{role:Role.MEMBER}}; type valid credentials.</t>
+  </si>
+  <si>
+    <t>login called once with valid credentials; router.push called with /member/dashboard.</t>
+  </si>
+  <si>
+    <t>TC-14</t>
+  </si>
+  <si>
+    <t>Successful login with an unrecognised role follows the switch default and navigates to login.</t>
+  </si>
+  <si>
+    <t>login resolves {success:true,data:{role:"UNKNOWN" as Role}}; type valid credentials.</t>
+  </si>
+  <si>
+    <t>login called once; router.push called with /login.</t>
+  </si>
+  <si>
+    <t>TC-15</t>
+  </si>
+  <si>
+    <t>Successful login result without session data does not navigate and shows no error alert.</t>
+  </si>
+  <si>
+    <t>login resolves {success:true,data:undefined}; type valid credentials.</t>
+  </si>
+  <si>
+    <t>login called once; router.push not called; no alert is visible.</t>
+  </si>
+  <si>
+    <t>TC-16</t>
+  </si>
+  <si>
+    <t>Failed login result shows server message and re-enables the submit button.</t>
+  </si>
+  <si>
+    <t>login resolves {success:false,message:"Invalid credentials"}; type valid credentials.</t>
+  </si>
+  <si>
+    <t>Alert contains Invalid credentials; Sign in button enabled; router.push not called.</t>
+  </si>
+  <si>
+    <t>TC-17</t>
+  </si>
+  <si>
+    <t>Failed login result with field errors renders server email and password field errors.</t>
+  </si>
+  <si>
+    <t>login resolves failed result with errors.email and errors.password; type valid credentials.</t>
+  </si>
+  <si>
+    <t>Server email and password error messages are visible; router.push not called.</t>
+  </si>
+  <si>
+    <t>TC-18</t>
+  </si>
+  <si>
+    <t>Pending login disables the submit button and changes the label to Signing in.</t>
+  </si>
+  <si>
+    <t>login returns a manually controlled unresolved promise; type valid credentials.</t>
+  </si>
+  <si>
+    <t>userEvent.click(Sign in) without resolving login.</t>
+  </si>
+  <si>
+    <t>Button is disabled; Signing in… text visible; Sign in text absent until cleanup resolves promise.</t>
+  </si>
+  <si>
+    <t>TC-19</t>
+  </si>
+  <si>
+    <t>After a server-side failure, a subsequent valid submission can succeed.</t>
+  </si>
+  <si>
+    <t>login first resolves failed Invalid credentials, then resolves success with MEMBER role; type valid credentials.</t>
+  </si>
+  <si>
+    <t>Click Sign in twice, waiting for the first alert before the second click.</t>
+  </si>
+  <si>
+    <t>First click shows Invalid credentials; second click pushes /member/dashboard; login called twice.</t>
   </si>
   <si>
     <t>Testing</t>
@@ -776,14 +846,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="50" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" ht="35" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -827,7 +897,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" ht="50" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" ht="65" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
@@ -857,7 +927,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" ht="125" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" ht="95" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>14</v>
       </c>
@@ -879,7 +949,7 @@
       </c>
       <c r="B13" s="2"/>
     </row>
-    <row r="14" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" ht="35" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>1</v>
       </c>
@@ -895,7 +965,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" ht="50" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" ht="35" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>1</v>
       </c>
@@ -911,12 +981,20 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" ht="50" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" ht="35" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>1</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="19" ht="35" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -933,11 +1011,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
-    <col min="3" max="6" width="80" customWidth="1"/>
+    <col min="3" max="4" width="80" customWidth="1"/>
+    <col min="5" max="5" width="77" customWidth="1"/>
+    <col min="6" max="6" width="80" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
   </cols>
   <sheetData>
@@ -946,232 +1026,232 @@
         <v>1</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" ht="65" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" ht="50" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="G3" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" ht="65" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="F4" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" ht="65" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" ht="50" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" ht="50" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>1</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" ht="50" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>1</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" ht="50" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>1</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" ht="50" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>67</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" ht="80" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>1</v>
       </c>
@@ -1185,13 +1265,220 @@
         <v>70</v>
       </c>
       <c r="E11" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="G11" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="G11" s="7" t="s">
-        <v>33</v>
+      <c r="C12" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1219,17 +1506,17 @@
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>73</v>
+        <v>110</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2" t="s">
-        <v>74</v>
+        <v>111</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>75</v>
+        <v>112</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
@@ -1241,40 +1528,40 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>76</v>
+        <v>113</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>77</v>
+        <v>114</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>78</v>
+        <v>115</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>79</v>
+        <v>116</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>80</v>
+        <v>117</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>81</v>
+        <v>118</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>82</v>
+        <v>119</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>83</v>
+        <v>120</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>77</v>
+        <v>114</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>78</v>
+        <v>115</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>79</v>
+        <v>116</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>80</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1282,40 +1569,40 @@
         <v>1</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>84</v>
+        <v>121</v>
       </c>
       <c r="C6" s="4">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D6" s="4">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E6" s="4">
         <v>0</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>85</v>
+        <v>122</v>
       </c>
       <c r="G6" s="4">
         <v>0</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>86</v>
+        <v>123</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>87</v>
+        <v>124</v>
       </c>
       <c r="J6" s="4">
         <v>0</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>88</v>
+        <v>125</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>88</v>
+        <v>125</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>88</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25"/>
@@ -1324,7 +1611,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>89</v>
+        <v>126</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>4</v>

</xml_diff>